<commit_message>
start new problem Array of Anagrams
</commit_message>
<xml_diff>
--- a/leetcode_tracker.xlsx
+++ b/leetcode_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EBOVES\Desktop\important papers\datastructure\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C60F2CB-E18B-4942-9A7E-E422F8371411}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F79D6A77-CF28-4DDE-AC89-614A102B184D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="59">
   <si>
     <t>Elvis's LeetCode Progress Tracker</t>
   </si>
@@ -136,9 +136,6 @@
     <t>String, Hash Table</t>
   </si>
   <si>
-    <t>125</t>
-  </si>
-  <si>
     <t>Topic/Category Statistics</t>
   </si>
   <si>
@@ -193,9 +190,6 @@
     <t>Binary Search</t>
   </si>
   <si>
-    <t>Skipped</t>
-  </si>
-  <si>
     <t>saved each char in a dict and add 1 every time y see a char in a string and then subtract one if that char is contained in the other string.</t>
   </si>
   <si>
@@ -209,6 +203,15 @@
   </si>
   <si>
     <t>need to learn more about how to interpret the problem.</t>
+  </si>
+  <si>
+    <t>Variables</t>
+  </si>
+  <si>
+    <t>Array of Anagrams</t>
+  </si>
+  <si>
+    <t>Working</t>
   </si>
 </sst>
 </file>
@@ -415,7 +418,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -468,11 +471,87 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="13">
+    <dxf>
+      <font>
+        <color theme="7" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="3" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -644,7 +723,7 @@
                   <c:v>Medium Problems</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1134,18 +1213,18 @@
         <v>32</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23">
-        <v>46126</v>
+        <v>46125</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>20</v>
@@ -1156,54 +1235,73 @@
       <c r="E5" s="7">
         <v>20</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" s="7"/>
+      <c r="F5" s="7">
+        <v>121</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>56</v>
+      </c>
       <c r="H5" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I5" s="7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="25">
+        <v>46126</v>
+      </c>
+      <c r="B6" s="24" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C6" s="10" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>52</v>
+        <v>58</v>
+      </c>
+      <c r="F6">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C6">
-    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Hard">
+    <cfRule type="containsText" dxfId="12" priority="5" operator="containsText" text="Hard">
       <formula>NOT(ISERROR(SEARCH("Hard",C2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Medium">
+    <cfRule type="containsText" dxfId="11" priority="6" operator="containsText" text="Medium">
       <formula>NOT(ISERROR(SEARCH("Medium",C2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="7" operator="containsText" text="Easy">
+    <cfRule type="containsText" dxfId="10" priority="8" operator="containsText" text="Easy">
       <formula>NOT(ISERROR(SEARCH("Easy",C2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D6">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Skipped">
+    <cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="Skipped">
       <formula>NOT(ISERROR(SEARCH("Skipped",D2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Reviewed">
+    <cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="Reviewed">
       <formula>NOT(ISERROR(SEARCH("Reviewed",D2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Stuck">
+    <cfRule type="containsText" dxfId="7" priority="4" operator="containsText" text="Stuck">
       <formula>NOT(ISERROR(SEARCH("Stuck",D2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <conditionalFormatting sqref="D6">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Working">
+      <formula>NOT(ISERROR(SEARCH("Working",D6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
     <dataValidation type="list" errorTitle="Invalid Difficulty" error="Please select Easy, Medium, or Hard" sqref="C2:C1000" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Easy,Medium,Hard"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorTitle="Invalid Status" error="Please select a valid status" sqref="D2:D1000" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" errorTitle="Invalid Status" error="Please select a valid status" sqref="D2:D5 D7:D1000" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Solved,Stuck,Reviewed,Skipped"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorTitle="Invalid Status" error="Please select a valid status" sqref="D6" xr:uid="{7B6D9C7E-5167-4F88-8D17-907A1AC10E12}">
+      <formula1>"Solved,Stuck,Reviewed,Skipped,Working"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1259,12 +1357,12 @@
     <row r="6" spans="1:6" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A6" s="18">
         <f>COUNTA('Problem Log'!A:A)-1</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" s="11"/>
       <c r="D6" s="20">
         <f>COUNTIF('Problem Log'!C:C,"Easy")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E6" s="11"/>
     </row>
@@ -1281,7 +1379,7 @@
     <row r="9" spans="1:6" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A9" s="15">
         <f>COUNTIF('Problem Log'!C:C,"Medium")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" s="11"/>
       <c r="D9" s="16">
@@ -1368,7 +1466,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -1376,86 +1474,86 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>20</v>
       </c>
       <c r="C2" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="8" t="s">
         <v>36</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
This is a new problem: Palindrome
</commit_message>
<xml_diff>
--- a/leetcode_tracker.xlsx
+++ b/leetcode_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EBOVES\Desktop\important papers\datastructure\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F79D6A77-CF28-4DDE-AC89-614A102B184D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DAF5B43-C829-422F-BE74-D801C4DF586D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -418,7 +418,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -446,6 +446,15 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -468,20 +477,14 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="7">
     <dxf>
       <font>
         <color theme="7" tint="-0.24994659260841701"/>
@@ -489,66 +492,6 @@
       <fill>
         <patternFill>
           <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="3" tint="-0.24994659260841701"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -630,16 +573,33 @@
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="1"/>
-  <c:style val="10"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
   <c:chart>
     <c:title>
       <c:tx>
         <c:rich>
-          <a:bodyPr/>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="75000"/>
+                    <a:lumOff val="25000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
@@ -649,6 +609,33 @@
         </c:rich>
       </c:tx>
       <c:overlay val="1"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="75000"/>
+                  <a:lumOff val="25000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -658,21 +645,23 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </c:spPr>
           <c:dPt>
             <c:idx val="0"/>
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="006100"/>
+                <a:schemeClr val="accent1"/>
               </a:solidFill>
               <a:ln>
-                <a:prstDash val="solid"/>
+                <a:noFill/>
               </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="20000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -685,11 +674,18 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="9C6500"/>
+                <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:ln>
-                <a:prstDash val="solid"/>
+                <a:noFill/>
               </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="20000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -702,11 +698,18 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="9C0006"/>
+                <a:schemeClr val="accent3"/>
               </a:solidFill>
               <a:ln>
-                <a:prstDash val="solid"/>
+                <a:noFill/>
               </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="20000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -714,6 +717,77 @@
               </c:ext>
             </c:extLst>
           </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:pattFill prst="pct75">
+                <a:fgClr>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="75000"/>
+                    <a:lumOff val="25000"/>
+                  </a:schemeClr>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="40000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="lt1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525">
+                  <a:solidFill>
+                    <a:schemeClr val="dk1">
+                      <a:lumMod val="50000"/>
+                      <a:lumOff val="50000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>Dashboard!$A$8:$A$10</c:f>
@@ -744,31 +818,753 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
+          <c:dLblPos val="ctr"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
           <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
+          <c:showPercent val="1"/>
           <c:showBubbleSize val="0"/>
           <c:showLeaderLines val="1"/>
         </c:dLbls>
         <c:firstSliceAng val="0"/>
       </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:overlay val="1"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="39000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="75000"/>
+                  <a:lumOff val="25000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="1"/>
   </c:chart>
+  <c:spPr>
+    <a:gradFill flip="none" rotWithShape="1">
+      <a:gsLst>
+        <a:gs pos="0">
+          <a:schemeClr val="lt1"/>
+        </a:gs>
+        <a:gs pos="39000">
+          <a:schemeClr val="lt1"/>
+        </a:gs>
+        <a:gs pos="100000">
+          <a:schemeClr val="lt1">
+            <a:lumMod val="75000"/>
+          </a:schemeClr>
+        </a:gs>
+      </a:gsLst>
+      <a:path path="circle">
+        <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+      </a:path>
+      <a:tileRect/>
+    </a:gradFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="25000"/>
+          <a:lumOff val="75000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
   <c:printSettings>
     <c:headerFooter/>
     <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="253">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200" cap="all" baseline="0"/>
+  </cs:categoryAxis>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:gradFill flip="none" rotWithShape="1">
+        <a:gsLst>
+          <a:gs pos="0">
+            <a:schemeClr val="lt1"/>
+          </a:gs>
+          <a:gs pos="39000">
+            <a:schemeClr val="lt1"/>
+          </a:gs>
+          <a:gs pos="100000">
+            <a:schemeClr val="lt1">
+              <a:lumMod val="75000"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:path path="circle">
+          <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+        </a:path>
+        <a:tileRect/>
+      </a:gradFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:pattFill prst="pct75">
+        <a:fgClr>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:fgClr>
+        <a:bgClr>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:bgClr>
+      </a:pattFill>
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:spPr>
+    <cs:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:pattFill prst="pct75">
+        <a:fgClr>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:fgClr>
+        <a:bgClr>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:bgClr>
+      </a:pattFill>
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:spPr>
+    <cs:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:effectLst>
+        <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="20000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:effectLst>
+        <a:outerShdw blurRad="254000" sx="102000" sy="102000" algn="ctr" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="20000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="31750" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:alpha val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr">
+          <a:alpha val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="50000"/>
+          <a:lumOff val="50000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="100000">
+              <a:schemeClr val="dk1">
+                <a:lumMod val="95000"/>
+                <a:lumOff val="5000"/>
+                <a:alpha val="42000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="0">
+              <a:schemeClr val="lt1">
+                <a:lumMod val="75000"/>
+                <a:alpha val="36000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="100000">
+              <a:schemeClr val="dk1">
+                <a:lumMod val="95000"/>
+                <a:lumOff val="5000"/>
+                <a:alpha val="42000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="0">
+              <a:schemeClr val="lt1">
+                <a:lumMod val="75000"/>
+                <a:alpha val="36000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1">
+          <a:lumMod val="95000"/>
+          <a:alpha val="39000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="31750" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1800" b="1" kern="1200" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1133,7 +1929,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="23">
+      <c r="A2" s="11">
         <v>46119</v>
       </c>
       <c r="B2" s="7" t="s">
@@ -1162,7 +1958,7 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23">
+      <c r="A3" s="11">
         <v>46120</v>
       </c>
       <c r="B3" s="7" t="s">
@@ -1191,7 +1987,7 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23">
+      <c r="A4" s="11">
         <v>46125</v>
       </c>
       <c r="B4" s="7" t="s">
@@ -1220,7 +2016,7 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="23">
+      <c r="A5" s="11">
         <v>46125</v>
       </c>
       <c r="B5" s="7" t="s">
@@ -1249,10 +2045,10 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="25">
+      <c r="A6" s="13">
         <v>46126</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="12" t="s">
         <v>57</v>
       </c>
       <c r="C6" s="10" t="s">
@@ -1261,30 +2057,33 @@
       <c r="D6" s="10" t="s">
         <v>58</v>
       </c>
+      <c r="E6" s="26">
+        <v>0</v>
+      </c>
       <c r="F6">
         <v>49</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C6">
-    <cfRule type="containsText" dxfId="12" priority="5" operator="containsText" text="Hard">
+    <cfRule type="containsText" dxfId="6" priority="5" operator="containsText" text="Hard">
       <formula>NOT(ISERROR(SEARCH("Hard",C2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="6" operator="containsText" text="Medium">
+    <cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="Medium">
       <formula>NOT(ISERROR(SEARCH("Medium",C2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="8" operator="containsText" text="Easy">
+    <cfRule type="containsText" dxfId="4" priority="8" operator="containsText" text="Easy">
       <formula>NOT(ISERROR(SEARCH("Easy",C2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D6">
-    <cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="Skipped">
+    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="Skipped">
       <formula>NOT(ISERROR(SEARCH("Skipped",D2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="Reviewed">
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Reviewed">
       <formula>NOT(ISERROR(SEARCH("Reviewed",D2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="4" operator="containsText" text="Stuck">
+    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="Stuck">
       <formula>NOT(ISERROR(SEARCH("Stuck",D2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1319,119 +2118,119 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
     </row>
     <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="D5" s="12" t="s">
+      <c r="B5" s="14"/>
+      <c r="D5" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="11"/>
+      <c r="E5" s="14"/>
     </row>
     <row r="6" spans="1:6" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="A6" s="18">
+      <c r="A6" s="21">
         <f>COUNTA('Problem Log'!A:A)-1</f>
         <v>5</v>
       </c>
-      <c r="B6" s="11"/>
-      <c r="D6" s="20">
+      <c r="B6" s="14"/>
+      <c r="D6" s="23">
         <f>COUNTIF('Problem Log'!C:C,"Easy")</f>
         <v>4</v>
       </c>
-      <c r="E6" s="11"/>
+      <c r="E6" s="14"/>
     </row>
     <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="11"/>
-      <c r="D8" s="19" t="s">
+      <c r="B8" s="14"/>
+      <c r="D8" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="11"/>
+      <c r="E8" s="14"/>
     </row>
     <row r="9" spans="1:6" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="A9" s="15">
+      <c r="A9" s="18">
         <f>COUNTIF('Problem Log'!C:C,"Medium")</f>
         <v>1</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="D9" s="16">
+      <c r="B9" s="14"/>
+      <c r="D9" s="19">
         <f>COUNTIF('Problem Log'!C:C,"Hard")</f>
         <v>0</v>
       </c>
-      <c r="E9" s="11"/>
+      <c r="E9" s="14"/>
     </row>
     <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -1465,12 +2264,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">

</xml_diff>

<commit_message>
Add new problem to solve Mayority Element
</commit_message>
<xml_diff>
--- a/leetcode_tracker.xlsx
+++ b/leetcode_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EBOVES\Desktop\important papers\datastructure\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DAF5B43-C829-422F-BE74-D801C4DF586D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB608ED6-0B67-4B68-ABA8-EB66DC1FA3BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="62">
   <si>
     <t>Elvis's LeetCode Progress Tracker</t>
   </si>
@@ -208,10 +208,19 @@
     <t>Variables</t>
   </si>
   <si>
-    <t>Array of Anagrams</t>
-  </si>
-  <si>
     <t>Working</t>
+  </si>
+  <si>
+    <t>Polidrome two pointers</t>
+  </si>
+  <si>
+    <t>has to ask claude since I've never done a two pointers but now I know to to solve it.</t>
+  </si>
+  <si>
+    <t>when dealing with two pointers, need a var for the start and one for the end; the last one using the len(s) -1. and need to check if they are in the middle of the list.</t>
+  </si>
+  <si>
+    <t>Majority Element</t>
   </si>
 </sst>
 </file>
@@ -376,7 +385,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -414,11 +423,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -479,6 +499,10 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -797,7 +821,7 @@
                   <c:v>Medium Problems</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1888,7 +1912,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2015,7 +2039,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11">
         <v>46125</v>
       </c>
@@ -2044,28 +2068,54 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13">
         <v>46126</v>
       </c>
       <c r="B6" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="26">
+        <v>10</v>
+      </c>
+      <c r="F6">
+        <v>125</v>
+      </c>
+      <c r="G6" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="H6" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="I6" s="26" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="27">
+        <v>46127</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="E6" s="26">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>49</v>
+      <c r="F7">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C2:C6">
+  <conditionalFormatting sqref="C2:C7">
     <cfRule type="containsText" dxfId="6" priority="5" operator="containsText" text="Hard">
       <formula>NOT(ISERROR(SEARCH("Hard",C2)))</formula>
     </cfRule>
@@ -2076,7 +2126,7 @@
       <formula>NOT(ISERROR(SEARCH("Easy",C2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D6">
+  <conditionalFormatting sqref="D2:D7">
     <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="Skipped">
       <formula>NOT(ISERROR(SEARCH("Skipped",D2)))</formula>
     </cfRule>
@@ -2087,7 +2137,7 @@
       <formula>NOT(ISERROR(SEARCH("Stuck",D2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D6">
+  <conditionalFormatting sqref="D6:D7">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Working">
       <formula>NOT(ISERROR(SEARCH("Working",D6)))</formula>
     </cfRule>
@@ -2096,13 +2146,16 @@
     <dataValidation type="list" errorTitle="Invalid Difficulty" error="Please select Easy, Medium, or Hard" sqref="C2:C1000" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Easy,Medium,Hard"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorTitle="Invalid Status" error="Please select a valid status" sqref="D2:D5 D7:D1000" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" errorTitle="Invalid Status" error="Please select a valid status" sqref="D2:D5 D8:D1000" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Solved,Stuck,Reviewed,Skipped"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorTitle="Invalid Status" error="Please select a valid status" sqref="D6" xr:uid="{7B6D9C7E-5167-4F88-8D17-907A1AC10E12}">
+    <dataValidation type="list" errorTitle="Invalid Status" error="Please select a valid status" sqref="D6:D7" xr:uid="{7B6D9C7E-5167-4F88-8D17-907A1AC10E12}">
       <formula1>"Solved,Stuck,Reviewed,Skipped,Working"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="B7" r:id="rId1" display="https://leetcode.com/problems/majority-element/" xr:uid="{3BFB7FC2-0744-426D-B43E-B468482D6735}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2156,12 +2209,12 @@
     <row r="6" spans="1:6" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A6" s="21">
         <f>COUNTA('Problem Log'!A:A)-1</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" s="14"/>
       <c r="D6" s="23">
         <f>COUNTIF('Problem Log'!C:C,"Easy")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E6" s="14"/>
     </row>
@@ -2178,7 +2231,7 @@
     <row r="9" spans="1:6" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A9" s="18">
         <f>COUNTIF('Problem Log'!C:C,"Medium")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B9" s="14"/>
       <c r="D9" s="19">

</xml_diff>